<commit_message>
Admin: edit data/showcase.xlsx via table editor
</commit_message>
<xml_diff>
--- a/data/showcase.xlsx
+++ b/data/showcase.xlsx
@@ -581,13 +581,13 @@
         <v>Shala Students Singing</v>
       </c>
       <c r="C7" t="str">
-        <v/>
+        <v>Hich Amuchi Prathana by Sankalp Marathi Students (Boston, MA)</v>
       </c>
       <c r="D7" t="str">
         <v>Competition</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>https://www.youtube.com/watch?v=OPvEpJOhSpY</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -596,10 +596,10 @@
         <v/>
       </c>
       <c r="H7" t="str">
-        <v/>
+        <v>Yes</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>